<commit_message>
v0.0.4 - Cohorts table and expenses_date field
</commit_message>
<xml_diff>
--- a/data/templates_data/other_marketing_costs_template.xlsx
+++ b/data/templates_data/other_marketing_costs_template.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -424,7 +424,7 @@
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>period_end</t>
+          <t>expenses_date</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">

</xml_diff>

<commit_message>
Update template Excel files: Replace 2013 dates with 2024 and 2014 dates with 2025
</commit_message>
<xml_diff>
--- a/data/templates_data/other_marketing_costs_template.xlsx
+++ b/data/templates_data/other_marketing_costs_template.xlsx
@@ -441,7 +441,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2013-03-31</t>
+          <t>2024-03-31</t>
         </is>
       </c>
       <c r="C2" t="n">
@@ -456,7 +456,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>2013-03-31</t>
+          <t>2024-03-31</t>
         </is>
       </c>
       <c r="C3" t="n">
@@ -471,7 +471,7 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>2013-03-31</t>
+          <t>2024-03-31</t>
         </is>
       </c>
       <c r="C4" t="n">
@@ -486,7 +486,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2013-03-31</t>
+          <t>2024-03-31</t>
         </is>
       </c>
       <c r="C5" t="n">
@@ -501,7 +501,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>2013-06-30</t>
+          <t>2024-06-30</t>
         </is>
       </c>
       <c r="C6" t="n">
@@ -516,7 +516,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>2013-06-30</t>
+          <t>2024-06-30</t>
         </is>
       </c>
       <c r="C7" t="n">
@@ -531,7 +531,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>2013-06-30</t>
+          <t>2024-06-30</t>
         </is>
       </c>
       <c r="C8" t="n">
@@ -546,7 +546,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>2013-06-30</t>
+          <t>2024-06-30</t>
         </is>
       </c>
       <c r="C9" t="n">
@@ -561,7 +561,7 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>2013-09-30</t>
+          <t>2024-09-30</t>
         </is>
       </c>
       <c r="C10" t="n">
@@ -576,7 +576,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>2013-09-30</t>
+          <t>2024-09-30</t>
         </is>
       </c>
       <c r="C11" t="n">
@@ -591,7 +591,7 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>2013-09-30</t>
+          <t>2024-09-30</t>
         </is>
       </c>
       <c r="C12" t="n">
@@ -606,7 +606,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>2013-09-30</t>
+          <t>2024-09-30</t>
         </is>
       </c>
       <c r="C13" t="n">
@@ -621,7 +621,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>2013-12-31</t>
+          <t>2024-12-31</t>
         </is>
       </c>
       <c r="C14" t="n">
@@ -636,7 +636,7 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>2013-12-31</t>
+          <t>2024-12-31</t>
         </is>
       </c>
       <c r="C15" t="n">
@@ -651,7 +651,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>2013-12-31</t>
+          <t>2024-12-31</t>
         </is>
       </c>
       <c r="C16" t="n">
@@ -666,7 +666,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>2013-12-31</t>
+          <t>2024-12-31</t>
         </is>
       </c>
       <c r="C17" t="n">
@@ -681,7 +681,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>2014-03-31</t>
+          <t>2025-03-31</t>
         </is>
       </c>
       <c r="C18" t="n">
@@ -696,7 +696,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>2014-03-31</t>
+          <t>2025-03-31</t>
         </is>
       </c>
       <c r="C19" t="n">
@@ -711,7 +711,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>2014-03-31</t>
+          <t>2025-03-31</t>
         </is>
       </c>
       <c r="C20" t="n">
@@ -726,7 +726,7 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>2014-03-31</t>
+          <t>2025-03-31</t>
         </is>
       </c>
       <c r="C21" t="n">
@@ -741,7 +741,7 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>2014-06-30</t>
+          <t>2025-06-30</t>
         </is>
       </c>
       <c r="C22" t="n">
@@ -756,7 +756,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>2014-06-30</t>
+          <t>2025-06-30</t>
         </is>
       </c>
       <c r="C23" t="n">
@@ -771,7 +771,7 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>2014-06-30</t>
+          <t>2025-06-30</t>
         </is>
       </c>
       <c r="C24" t="n">
@@ -786,7 +786,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2014-06-30</t>
+          <t>2025-06-30</t>
         </is>
       </c>
       <c r="C25" t="n">
@@ -801,7 +801,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>2014-09-30</t>
+          <t>2025-09-30</t>
         </is>
       </c>
       <c r="C26" t="n">
@@ -816,7 +816,7 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>2014-09-30</t>
+          <t>2025-09-30</t>
         </is>
       </c>
       <c r="C27" t="n">
@@ -831,7 +831,7 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>2014-09-30</t>
+          <t>2025-09-30</t>
         </is>
       </c>
       <c r="C28" t="n">
@@ -846,7 +846,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>2014-09-30</t>
+          <t>2025-09-30</t>
         </is>
       </c>
       <c r="C29" t="n">
@@ -861,7 +861,7 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>2014-12-31</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="C30" t="n">
@@ -876,7 +876,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>2014-12-31</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="C31" t="n">
@@ -891,7 +891,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>2014-12-31</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="C32" t="n">
@@ -906,7 +906,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>2014-12-31</t>
+          <t>2025-12-31</t>
         </is>
       </c>
       <c r="C33" t="n">

</xml_diff>